<commit_message>
add productmatrix mtxcode var
</commit_message>
<xml_diff>
--- a/app/tests/output_MC_database.xlsx
+++ b/app/tests/output_MC_database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hoend008\OneDrive - WageningenUR\DEVELOPMENT\mc-api\app\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E830B370-466D-4040-8726-A023A2CA8D1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D0E3223-78A5-42CB-9D2D-93CE56BFC52E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{491A62C4-C058-41B1-B986-FDA3D06E3D52}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
   <si>
     <t>team_id</t>
   </si>
@@ -122,12 +122,6 @@
   </si>
   <si>
     <t>e02_sampmatcode4_nl</t>
-  </si>
-  <si>
-    <t>product/matrix code</t>
-  </si>
-  <si>
-    <t>mtx_code</t>
   </si>
   <si>
     <t>substance group</t>
@@ -345,6 +339,9 @@
   </si>
   <si>
     <t>updated_at</t>
+  </si>
+  <si>
+    <t>productmatrix_mtx_code</t>
   </si>
 </sst>
 </file>
@@ -405,18 +402,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -483,27 +474,24 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="1" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="1" fontId="6" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="6" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -848,7 +836,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A3FEA90-3D3B-48BA-99C0-69CCF6614005}">
-  <dimension ref="A1:BJ1"/>
+  <dimension ref="A1:BI1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.77734375" bestFit="1" customWidth="1"/>
@@ -871,55 +859,54 @@
     <col min="18" max="18" width="20.88671875" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="20.44140625" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="14.21875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="12" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="11" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="44" max="45" width="3.6640625" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="6.77734375" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="28.6640625" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="12" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="36.33203125" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="31" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="15.21875" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="20.88671875" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="12" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="11" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="43" max="44" width="3.6640625" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="6.77734375" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="12" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="36.33203125" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="31" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="20.88671875" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="10.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:62" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:61" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>1</v>
@@ -972,134 +959,131 @@
       <c r="S1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="T1" s="5" t="s">
+      <c r="T1" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="U1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="U1" s="5" t="s">
+      <c r="V1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="X1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="Y1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="Y1" s="3" t="s">
+      <c r="Z1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="AA1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AB1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="AB1" s="3" t="s">
+      <c r="AC1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AD1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AD1" s="3" t="s">
+      <c r="AE1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="AE1" s="6" t="s">
+      <c r="AF1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="AF1" s="3" t="s">
+      <c r="AG1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="AG1" s="3" t="s">
+      <c r="AH1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="AH1" s="3" t="s">
+      <c r="AI1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="AI1" s="3" t="s">
+      <c r="AJ1" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="AJ1" s="3" t="s">
+      <c r="AK1" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="AK1" s="3" t="s">
+      <c r="AL1" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="AL1" s="3" t="s">
+      <c r="AM1" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="AM1" s="3" t="s">
+      <c r="AN1" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="AN1" s="3" t="s">
+      <c r="AO1" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="AO1" s="3" t="s">
+      <c r="AP1" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="AP1" s="3" t="s">
+      <c r="AQ1" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="AQ1" s="3" t="s">
+      <c r="AR1" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="AR1" s="3" t="s">
+      <c r="AS1" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="AS1" s="3" t="s">
+      <c r="AT1" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="AT1" s="3" t="s">
+      <c r="AU1" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="AU1" s="3" t="s">
+      <c r="AV1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="AV1" s="3" t="s">
+      <c r="AW1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="AW1" s="6" t="s">
+      <c r="AX1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="AX1" s="6" t="s">
+      <c r="AY1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="AY1" s="6" t="s">
+      <c r="AZ1" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="AZ1" s="6" t="s">
+      <c r="BA1" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="BA1" s="3" t="s">
+      <c r="BB1" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="BB1" s="4" t="s">
+      <c r="BC1" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="BC1" s="3" t="s">
+      <c r="BD1" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="BD1" s="3" t="s">
+      <c r="BE1" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="BE1" s="3" t="s">
+      <c r="BF1" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="BF1" s="3" t="s">
+      <c r="BG1" s="3" t="s">
         <v>56</v>
-      </c>
-      <c r="BG1" s="3" t="s">
-        <v>57</v>
       </c>
       <c r="BH1" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="BI1" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="BJ1" s="7" t="s">
-        <v>61</v>
+      <c r="BI1" s="6" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>